<commit_message>
Fase 2: sincroniza Base de datos y calidad con la version del 23-10
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/calidad/Casos de Prueba.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/calidad/Casos de Prueba.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos de Prueba'!$A$1:$I$247</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos de Prueba'!$A$1:$I$248</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Gestor SSCC App · actualizado el 13-10-2026 13:01:16 · generado por el auditor automático</t>
+          <t>Volvo Dashboard App · actualizado el 22-10-2026 12:36:02 · generado por el auditor automático</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Cobertura por módulo (246 casos en total)</t>
+          <t>Cobertura por módulo (247 casos en total)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n"/>
@@ -697,7 +697,7 @@
         <v>27</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>0</v>
@@ -718,7 +718,7 @@
         <v>20</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>0</v>
@@ -823,7 +823,7 @@
         <v>6</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D23" s="13" t="n">
         <v>0</v>
@@ -1078,11 +1078,11 @@
         <v>125</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>Todo aprobado</t>
+        <v>2</v>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>Con fallas</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I247"/>
+  <dimension ref="A1:I248"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H2" s="14" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Problema 1 (post-migracion a LogApp.csv): tras una sincronizacion RM_CONTRATOS que genera cambios, el historial (LogApp.csv + DataManager.df_logs) debe quedar actualizado y Historial debe refrescarse solo, sin que el usuario tenga que presionar 'Actualizar'. La lectura de LogApp.csv debe ocurrir en el hilo de fondo (RMReporteSyncWorker), no en el hilo principal.</t>
+          <t>Problema 1 (post-migracion a LogApp.csv): tras una sincronizacion RM_JAVI que genera cambios, el historial (LogApp.csv + DataManager.df_logs) debe quedar actualizado y Historial debe refrescarse solo, sin que el usuario tenga que presionar 'Actualizar'. La lectura de LogApp.csv debe ocurrir en el hilo de fondo (RMJaviSyncWorker), no en el hilo principal.</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -1551,21 +1551,21 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMReporteSyncActualizaHistorial' (archivo test_comercial.py). 3) Pruebas incluidas: boton actualizar manual de historial sigue funcionando; historial no recibe filas tras sincronizar; sync actualiza datamanager sin emitir logs updated ni data ready; sync ya no escribe logapp csv.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMJaviSyncActualizaHistorial' (archivo test_comercial.py). 3) Pruebas incluidas: boton actualizar manual de historial sigue funcionando; historial no recibe filas tras sincronizar; sync actualiza datamanager sin emitir logs updated ni data ready; sync ya no escribe logapp csv.</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Las 4 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Problema 1 (post-migracion a LogApp.csv): tras una sincronizacion
-RM_CONTRATOS que genera cambios, el historial (LogApp.csv + DataManager.df_logs)
+RM_JAVI que genera cambios, el historial (LogApp.csv + DataManager.df_logs)
 debe quedar actualizado y Historial debe refrescarse solo, sin que el
 usuario tenga que presionar 'Actualizar'. La lectura de LogApp.csv debe
-ocurrir en el hilo de fondo (RMReporteSyncWorker), no en el hilo principal.</t>
+ocurrir en el hilo de fondo (RMJaviSyncWorker), no en el hilo principal.</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H3" s="14" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-053, CP-1219_CP-1221 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMReporteSyncActualizaHistorial.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-053, CP-1219_CP-1221 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMJaviSyncActualizaHistorial.</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H5" s="14" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H8" s="14" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 11 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 11 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H10" s="14" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H11" s="14" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H20" s="14" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
@@ -2875,7 +2875,7 @@
     <row r="31" ht="112" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>CP-122_CP-130</t>
+          <t>CP-122, CP-124_CP-130, CP-1431</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestContactos' (archivo test_contactos.py). 3) Pruebas incluidas: 01 carga datos falsos; 02 filtros lista checkbox; 03 edicion formato y llave original; 04 guardado asincrono; 05 eliminacion llave compuesta; 06 dialogo agregar autocompletado validacion y get data; … (y 3 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestContactos' (archivo test_contactos.py). 3) Pruebas incluidas: 01 carga datos falsos; 02 lista de flotas abre sus contactos; 03 edicion formato y llave original; 04 guardado asincrono; 05 eliminacion llave compuesta; 06 dialogo agregar autocompletado validacion y get data; … (y 3 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-122_CP-130 del Reporte de Ejecución. Test automatizado: src/tests/test_contactos.py::TestContactos.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-122, CP-124_CP-130, CP-1431 del Reporte de Ejecución. Test automatizado: src/tests/test_contactos.py::TestContactos.</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
@@ -3119,7 +3119,7 @@
     <row r="36" ht="98.5" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>CP-196_CP-201</t>
+          <t>CP-196_CP-198, CP-200_CP-201, CP-1433</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestObtenerConfiguracionPlantilla' (archivo test_mail_service.py). 3) Pruebas incluidas: asuntos no cambiaron; cada plantilla tiene asunto constructor e imagenes; constructor produce html; cubre las siete plantillas actuales; imagenes cid no cambiaron; nombre no reconocido devuelve none.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestObtenerConfiguracionPlantilla' (archivo test_mail_service.py). 3) Pruebas incluidas: asuntos no cambiaron; cada plantilla tiene asunto constructor e imagenes; constructor produce html; cubre las plantillas actuales; imagenes cid no cambiaron; nombre no reconocido devuelve none.</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-196_CP-201 del Reporte de Ejecución. Test automatizado: src/tests/test_mail_service.py::TestObtenerConfiguracionPlantilla.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-196_CP-198, CP-200_CP-201, CP-1433 del Reporte de Ejecución. Test automatizado: src/tests/test_mail_service.py::TestObtenerConfiguracionPlantilla.</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H39" s="14" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H40" s="14" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H42" s="14" t="inlineStr">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H43" s="14" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H44" s="14" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H45" s="14" t="inlineStr">
@@ -3637,7 +3637,7 @@
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestAppTableWidgetMenuEliminados' (archivo test_table_sorting.py). 3) Pruebas incluidas: restaurar fila esta deshabilitada.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestVolvoTableWidgetMenuEliminados' (archivo test_table_sorting.py). 3) Pruebas incluidas: restaurar fila esta deshabilitada.</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H46" s="14" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="I46" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-294 del Reporte de Ejecución. Test automatizado: src/tests/test_table_sorting.py::TestAppTableWidgetMenuEliminados.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-294 del Reporte de Ejecución. Test automatizado: src/tests/test_table_sorting.py::TestVolvoTableWidgetMenuEliminados.</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Pruebas puras (sin Excel/DataManager) del ordenamiento tipo Excel agregado a AppTableWidget: apply_sort() y el ciclo asc -&gt; desc -&gt; orden original disparado por clic de encabezado.</t>
+          <t>Pruebas puras (sin Excel/DataManager) del ordenamiento tipo Excel agregado a VolvoTableWidget: apply_sort() y el ciclo asc -&gt; desc -&gt; orden original disparado por clic de encabezado.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -3687,19 +3687,19 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestAppTableWidgetSorting' (archivo test_table_sorting.py). 3) Pruebas incluidas: columna ordenada ya no existe no lanza error; combinacion filtro y orden; elegir otra columna en el menu reemplaza el orden activo; orden persiste entre llamadas sucesivas con distintos df; ordenamiento ascendente texto; ordenamiento descendente texto; … (y 5 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestVolvoTableWidgetSorting' (archivo test_table_sorting.py). 3) Pruebas incluidas: columna ordenada ya no existe no lanza error; combinacion filtro y orden; elegir otra columna en el menu reemplaza el orden activo; orden persiste entre llamadas sucesivas con distintos df; ordenamiento ascendente texto; ordenamiento descendente texto; … (y 5 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Las 11 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Pruebas puras (sin Excel/DataManager) del ordenamiento tipo Excel
-agregado a AppTableWidget: apply_sort() y el ciclo asc -&gt; desc -&gt;
+agregado a VolvoTableWidget: apply_sort() y el ciclo asc -&gt; desc -&gt;
 orden original disparado por clic de encabezado.</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 11 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 11 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H47" s="14" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="I47" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-297_CP-305, CP-477_CP-478 del Reporte de Ejecución. Test automatizado: src/tests/test_table_sorting.py::TestAppTableWidgetSorting.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-297_CP-305, CP-477_CP-478 del Reporte de Ejecución. Test automatizado: src/tests/test_table_sorting.py::TestVolvoTableWidgetSorting.</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H48" s="14" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H49" s="14" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H50" s="14" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H51" s="14" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H52" s="14" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H53" s="14" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H54" s="14" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H55" s="14" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H56" s="14" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H57" s="14" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H58" s="14" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H59" s="14" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 16 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 16 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H60" s="14" t="inlineStr">
@@ -4390,14 +4390,14 @@
 (datetime/Timestamp) se convertia a string ISO ANTES de calcular_termino,
 y esta la reparseaba con pd.to_datetime(format='mixed', dayfirst=True),
 lo que intercambiaba dia y mes cuando ambos eran &lt;=12. Confirmado con
-datos reales de RM_CONTRATOS/PruebasFM (Fase C): ~60% de los registros con
+datos reales de RM_JAVI/PruebasFM (Fase C): ~60% de los registros con
 duracion numerica quedaban con TÉRMINO CONTRATO incorrecto en cada
 load/reload/sync.</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 23 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 23 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H61" s="14" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H62" s="14" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H63" s="14" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H64" s="14" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H65" s="14" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H66" s="14" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H67" s="14" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H68" s="14" t="inlineStr">
@@ -4783,7 +4783,7 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H69" s="14" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H70" s="14" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H71" s="14" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H72" s="14" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H73" s="14" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H74" s="14" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H75" s="14" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H76" s="14" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H77" s="14" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H78" s="14" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H79" s="14" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>El escape hatch BRAND_SKIP_QUALITY_SYNC debe omitir todo sin tocar ningun archivo.</t>
+          <t>El escape hatch VOLVO_SKIP_QUALITY_SYNC debe omitir todo sin tocar ningun archivo.</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -5306,13 +5306,13 @@
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>Las 1 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: El escape hatch BRAND_SKIP_QUALITY_SYNC debe omitir todo sin tocar
+          <t>Las 1 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: El escape hatch VOLVO_SKIP_QUALITY_SYNC debe omitir todo sin tocar
 ningun archivo.</t>
         </is>
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H80" s="14" t="inlineStr">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 25 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 25 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H81" s="14" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H82" s="14" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H83" s="14" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H84" s="14" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H85" s="14" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H86" s="14" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H87" s="14" t="inlineStr">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 14 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 14 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H88" s="14" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H89" s="14" t="inlineStr">
@@ -5875,7 +5875,7 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H91" s="14" t="inlineStr">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H94" s="14" t="inlineStr">
@@ -6089,14 +6089,14 @@
 COLUMNAS_UNIDADES_VISIBLES: CDB y Flota VC quedan fuera de esa tabla a
 pedido explícito (se siguen usando internamente para filtrar por CDB en
 la caja derecha). VIN también queda fuera
-de la vista desde el 10-09-2026 (a pedido de la contraparte comercial) pero se conserva en
+de la vista desde el 10-09-2026 (a pedido de Javiera) pero se conserva en
 COLUMNAS_UNIDADES y COLUMNAS_BUSQUEDA_UNIDADES -- ver
 TestAplicarBusquedaUnidades para la búsqueda por VIN oculto.</t>
         </is>
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H95" s="14" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H96" s="14" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H98" s="14" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H99" s="14" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H100" s="14" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H101" s="14" t="inlineStr">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H102" s="14" t="inlineStr">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>Bug real reportado: al abrir Comercial con el Excel real (columnas reducidas de 34 a 33 respecto a la última vez que se guardó el estado del header con AppTableWidget.set_table_id), Qt seguía pidiendo headerData(33, ...) -- fuera de rango para un DataFrame de 33 columnas -- y PandasTableModel.headerData() indexaba directo sobre self._df.columns sin validar el rango, crasheando con IndexError.</t>
+          <t>Bug real reportado: al abrir Comercial con el Excel real (columnas reducidas de 34 a 33 respecto a la última vez que se guardó el estado del header con VolvoTableWidget.set_table_id), Qt seguía pidiendo headerData(33, ...) -- fuera de rango para un DataFrame de 33 columnas -- y PandasTableModel.headerData() indexaba directo sobre self._df.columns sin validar el rango, crasheando con IndexError.</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
@@ -6500,7 +6500,7 @@
         <is>
           <t>Las 3 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Bug real reportado: al abrir Comercial con el Excel real (columnas
 reducidas de 34 a 33 respecto a la última vez que se guardó el estado
-del header con AppTableWidget.set_table_id), Qt seguía pidiendo
+del header con VolvoTableWidget.set_table_id), Qt seguía pidiendo
 headerData(33, ...) -- fuera de rango para un DataFrame de 33 columnas
 -- y PandasTableModel.headerData() indexaba directo sobre
 self._df.columns sin validar el rango, crasheando con IndexError.</t>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H103" s="14" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="C104" s="9" t="inlineStr">
         <is>
-          <t>AppTableWidget.set_table_id(): si el estado de columnas guardado en QSettings quedó con más columnas de las que tiene el modelo actual -- p.ej. el Excel real perdió una columna desde la última vez que se guardó ese estado -- restaurarlo no debe dejar el header con secciones "fantasma" (más allá de las columnas reales) ni volver a crashear headerData() para ninguna sección del header resultante.</t>
+          <t>VolvoTableWidget.set_table_id(): si el estado de columnas guardado en QSettings quedó con más columnas de las que tiene el modelo actual -- p.ej. el Excel real perdió una columna desde la última vez que se guardó ese estado -- restaurarlo no debe dejar el header con secciones "fantasma" (más allá de las columnas reales) ni volver a crashear headerData() para ninguna sección del header resultante.</t>
         </is>
       </c>
       <c r="D104" s="9" t="inlineStr">
@@ -6550,7 +6550,7 @@
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Las 1 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: AppTableWidget.set_table_id(): si el estado de columnas guardado en
+          <t>Las 1 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: VolvoTableWidget.set_table_id(): si el estado de columnas guardado en
 QSettings quedó con más columnas de las que tiene el modelo actual --
 p.ej. el Excel real perdió una columna desde la última vez que se
 guardó ese estado -- restaurarlo no debe dejar el header con secciones
@@ -6560,7 +6560,7 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H104" s="14" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>Cubre el esquema explícito de columnas de RMReporteSyncWorker (RM_CONTRATOS_COLUMNAS_AUTORIZADAS / PRUEBAS_FM_COLUMNAS_LOCALES / COLUMNAS_TECNICAS_SYNC): la sincronización ya no debe depender de list(df_pruebas.columns) para decidir qué columnas del RM sobreviven, ni preservar columnas locales legacy no autorizadas.</t>
+          <t>Cubre el esquema explícito de columnas de RMJaviSyncWorker (RM_JAVI_COLUMNAS_AUTORIZADAS / PRUEBAS_FM_COLUMNAS_LOCALES / COLUMNAS_TECNICAS_SYNC): la sincronización ya no debe depender de list(df_pruebas.columns) para decidir qué columnas del RM sobreviven, ni preservar columnas locales legacy no autorizadas.</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
@@ -6597,20 +6597,20 @@
       </c>
       <c r="E105" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMReporteSyncColumnasAutorizadas' (archivo test_comercial.py). 3) Pruebas incluidas: alias de nombres siguen funcionando; celda vacia termina como guion y cero se conserva; columnas legacy de contacto dejan de persistirse; columnas no autorizadas del rm no entran; duracion existente en pruebasfm se pierde si rm llega vacia; duracion mensual del rm reemplaza duracion y termino antiguos; … (y 8 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMJaviSyncColumnasAutorizadas' (archivo test_comercial.py). 3) Pruebas incluidas: alias de nombres siguen funcionando; celda vacia termina como guion y cero se conserva; columnas legacy de contacto dejan de persistirse; columnas no autorizadas del rm no entran; duracion existente en pruebasfm se pierde si rm llega vacia; duracion mensual del rm reemplaza duracion y termino antiguos; … (y 8 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Las 14 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Cubre el esquema explícito de columnas de RMReporteSyncWorker
-(RM_CONTRATOS_COLUMNAS_AUTORIZADAS / PRUEBAS_FM_COLUMNAS_LOCALES / COLUMNAS_TECNICAS_SYNC):
+          <t>Las 14 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Cubre el esquema explícito de columnas de RMJaviSyncWorker
+(RM_JAVI_COLUMNAS_AUTORIZADAS / PRUEBAS_FM_COLUMNAS_LOCALES / COLUMNAS_TECNICAS_SYNC):
 la sincronización ya no debe depender de list(df_pruebas.columns) para decidir qué
 columnas del RM sobreviven, ni preservar columnas locales legacy no autorizadas.</t>
         </is>
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 14 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 14 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H105" s="14" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="I105" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-482_CP-485, CP-487_CP-491, CP-690_CP-693, CP-1222 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMReporteSyncColumnasAutorizadas.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-482_CP-485, CP-487_CP-491, CP-690_CP-693, CP-1222 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMJaviSyncColumnasAutorizadas.</t>
         </is>
       </c>
     </row>
@@ -6662,7 +6662,7 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H106" s="14" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 24 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 24 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H107" s="14" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>ETAPA GESTIÓN debe calcularse dentro de DataFrameFormatter.clean(), no depender del valor que venga escrito manualmente desde RM_CONTRATOS. Prioridad 1: TIPO DE FACTURACION contiene SIN REGISTRO -&gt; COMERCIAL, sin importar ESTADO COMERCIAL. Prioridad 2: ESTADO COMERCIAL -&gt; ETAPA GESTIÓN via ESTADO_COMERCIAL_ETAPA_MAP. Si ESTADO COMERCIAL no esta contemplado en el mapa, se conserva el valor de ETAPA GESTIÓN que ya traia…</t>
+          <t>ETAPA GESTIÓN debe calcularse dentro de DataFrameFormatter.clean(), no depender del valor que venga escrito manualmente desde RM_JAVI. Prioridad 1: TIPO DE FACTURACION contiene SIN REGISTRO -&gt; COMERCIAL, sin importar ESTADO COMERCIAL. Prioridad 2: ESTADO COMERCIAL -&gt; ETAPA GESTIÓN via ESTADO_COMERCIAL_ETAPA_MAP. Si ESTADO COMERCIAL no esta contemplado en el mapa, se conserva el valor de ETAPA GESTIÓN que ya traia…</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
@@ -6760,7 +6760,7 @@
       <c r="F108" s="9" t="inlineStr">
         <is>
           <t>Las 21 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: ETAPA GESTIÓN debe calcularse dentro de DataFrameFormatter.clean(), no
-depender del valor que venga escrito manualmente desde RM_CONTRATOS.
+depender del valor que venga escrito manualmente desde RM_JAVI.
 Orden de prioridades (reordenado 25-09-2026, a pedido explícito del
 usuario -- "la matriz de ESTADO COMERCIAL manda a todas las demás";
 antes SIN REGISTRO/FACTURACIÓN MANUAL tenían la prioridad más alta,
@@ -6781,7 +6781,7 @@
       </c>
       <c r="G108" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 21 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 21 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H108" s="14" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H109" s="14" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="C110" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: en Vista Completa (_ComercialModuleLegacy), al editar manualmente FORMA DE CONTRATO a 'Sin Contrato', se limpian a '-' TIPO DE SERVICIO, INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO CONTRATO de esa fila. Se dispara únicamente en ComercialModule.on_item_edited() (mismo mecanismo de pending_changes que cualquier otra edición manual); no hay limpieza retroactiva de filas ya en ESTADO COME…</t>
+          <t>Regla confirmada con Javiera: en Vista Completa (_ComercialModuleLegacy), al editar manualmente FORMA DE CONTRATO a 'Sin Contrato', se limpian a '-' TIPO DE SERVICIO, INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO CONTRATO de esa fila. Se dispara únicamente en ComercialModule.on_item_edited() (mismo mecanismo de pending_changes que cualquier otra edición manual); no hay limpieza retroactiva de filas ya en ESTADO COME…</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="F110" s="9" t="inlineStr">
         <is>
-          <t>Las 9 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con la contraparte comercial: en Vista Completa (_ComercialModuleLegacy),
+          <t>Las 9 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con Javiera: en Vista Completa (_ComercialModuleLegacy),
 al editar manualmente FORMA DE CONTRATO a 'Sin Contrato', se limpian a
 '-' TIPO DE SERVICIO, INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO
 CONTRATO de esa fila. Se dispara únicamente en
@@ -6883,7 +6883,7 @@
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H110" s="14" t="inlineStr">
@@ -6910,7 +6910,7 @@
       </c>
       <c r="C111" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: al editar FORMA DE CONTRATO a 'Sin Contrato' en Vista Completa, se limpian a '-' TIPO DE SERVICIO, INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO CONTRATO. Función pura: no conoce pending_changes, PyQt ni el DataFrame completo (eso es responsabilidad de comercial.py::on_item_edited).</t>
+          <t>Regla confirmada con Javiera: al editar FORMA DE CONTRATO a 'Sin Contrato' en Vista Completa, se limpian a '-' TIPO DE SERVICIO, INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO CONTRATO. Función pura: no conoce pending_changes, PyQt ni el DataFrame completo (eso es responsabilidad de comercial.py::on_item_edited).</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
@@ -6925,7 +6925,7 @@
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>Las 8 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con la contraparte comercial: al editar FORMA DE CONTRATO a
+          <t>Las 8 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con Javiera: al editar FORMA DE CONTRATO a
 'Sin Contrato' en Vista Completa, se limpian a '-' TIPO DE SERVICIO,
 INICIO CONTRATO, DURACIÓN (MESES) y TÉRMINO CONTRATO. Función pura: no
 conoce pending_changes, PyQt ni el DataFrame completo (eso es
@@ -6934,7 +6934,7 @@
       </c>
       <c r="G111" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H111" s="14" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="G112" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H112" s="14" t="inlineStr">
@@ -7037,7 +7037,7 @@
       </c>
       <c r="G113" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H113" s="14" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="G114" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H114" s="14" t="inlineStr">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="G115" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H115" s="14" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="G116" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H116" s="14" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="G117" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H117" s="14" t="inlineStr">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="G118" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H118" s="14" t="inlineStr">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="G119" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H119" s="14" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="G120" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H120" s="14" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="G121" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H121" s="14" t="inlineStr">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="G122" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H122" s="14" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="G123" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H123" s="14" t="inlineStr">
@@ -7570,7 +7570,7 @@
       </c>
       <c r="G124" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H124" s="14" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="G125" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H125" s="14" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="G126" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H126" s="14" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="G127" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H127" s="14" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="G128" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H128" s="14" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="G129" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H129" s="14" t="inlineStr">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="G130" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H130" s="14" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="G131" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H131" s="14" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="G132" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H132" s="14" t="inlineStr">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="C133" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: 'ACTIVO' es un error de digitacion, no un ESTADO COMERCIAL valido -- el dato correcto es 'VIGENTE'. La correccion debe ocurrir en RMReporteSyncWorker, ANTES de escribir a PruebasFM, sin alterar ningun otro valor de la columna.</t>
+          <t>Regla confirmada con Javiera: 'ACTIVO' es un error de digitacion, no un ESTADO COMERCIAL valido -- el dato correcto es 'VIGENTE'. La correccion debe ocurrir en RMJaviSyncWorker, ANTES de escribir a PruebasFM, sin alterar ningun otro valor de la columna.</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
@@ -8048,20 +8048,20 @@
       </c>
       <c r="E133" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMReporteSyncNormalizaEstadoComercial' (archivo test_comercial.py). 3) Pruebas incluidas: activo minusculas tambien se normaliza; activo se normaliza a vigente; baja permanece baja; baja solicitada no se altera; revisar permanece revisar; vencido permanece vencido; … (y 1 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMJaviSyncNormalizaEstadoComercial' (archivo test_comercial.py). 3) Pruebas incluidas: activo minusculas tambien se normaliza; activo se normaliza a vigente; baja permanece baja; baja solicitada no se altera; revisar permanece revisar; vencido permanece vencido; … (y 1 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>Las 7 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con la contraparte comercial: 'ACTIVO' es un error de digitacion, no
+          <t>Las 7 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con Javiera: 'ACTIVO' es un error de digitacion, no
 un ESTADO COMERCIAL valido -- el dato correcto es 'VIGENTE'. La
-correccion debe ocurrir en RMReporteSyncWorker, ANTES de escribir a
+correccion debe ocurrir en RMJaviSyncWorker, ANTES de escribir a
 PruebasFM, sin alterar ningun otro valor de la columna.</t>
         </is>
       </c>
       <c r="G133" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H133" s="14" t="inlineStr">
@@ -8071,14 +8071,14 @@
       </c>
       <c r="I133" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-694_CP-700 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMReporteSyncNormalizaEstadoComercial.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-694_CP-700 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMJaviSyncNormalizaEstadoComercial.</t>
         </is>
       </c>
     </row>
     <row r="134" ht="125.5" customHeight="1">
       <c r="A134" s="10" t="inlineStr">
         <is>
-          <t>CP-701_CP-705</t>
+          <t>CP-701_CP-702, CP-704_CP-705, CP-1426</t>
         </is>
       </c>
       <c r="B134" s="9" t="inlineStr">
@@ -8098,7 +8098,7 @@
       </c>
       <c r="E134" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestReconciliacionEstadoExpiredAlGuardarEnComercial' (archivo test_comercial.py). 3) Pruebas incluidas: edicion no guardada no genera caso; expired a running guardado resuelve el caso; expired a terminated guardado resuelve el caso y limpia campos; no duplica si se guarda dos veces sin cambiar el estado; running a expired guardado genera caso en revision cm.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestReconciliacionEstadoExpiredAlGuardarEnComercial' (archivo test_comercial.py). 3) Pruebas incluidas: edicion no guardada no genera caso; expired a running guardado resuelve el caso; expired a terminated guardado resuelve el caso y conserva campos; no duplica si se guarda dos veces sin cambiar el estado; running a expired guardado genera caso en revision cm.</t>
         </is>
       </c>
       <c r="F134" s="9" t="inlineStr">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="G134" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H134" s="14" t="inlineStr">
@@ -8121,14 +8121,14 @@
       </c>
       <c r="I134" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-701_CP-705 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestReconciliacionEstadoExpiredAlGuardarEnComercial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="152.5" customHeight="1">
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-701_CP-702, CP-704_CP-705, CP-1426 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestReconciliacionEstadoExpiredAlGuardarEnComercial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="98.5" customHeight="1">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>CP-706_CP-708</t>
+          <t>CP-1427_CP-1428</t>
         </is>
       </c>
       <c r="B135" s="9" t="inlineStr">
@@ -8148,21 +8148,19 @@
       </c>
       <c r="E135" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestReglaTerminatedCm' (archivo test_comercial.py). 3) Pruebas incluidas: expired a terminated limpia cinco campos; running a terminated limpia cinco campos; terminated a otro valor no restaura datos.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestReglaTerminatedCm' (archivo test_comercial.py). 3) Pruebas incluidas: expired a terminated conserva datos del cm; running a terminated conserva datos del cm.</t>
         </is>
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>Las 3 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada: en Vista Completa (_ComercialModuleLegacy), al
-editar manualmente ESTADO DEL CM a 'Terminated', se limpian a '-'
-N CONTRATO 3PC, FECHA INICIO CM, FECHA TERMINO CM, TIPO DE CM y PAGO CM
-de esa fila. Mismo mecanismo de pending_changes que cualquier otra
-edición manual (ver TestReglaSinContrato); no hay regla inversa.</t>
+          <t>Las 2 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: En Vista Completa (_ComercialModuleLegacy), al editar manualmente
+ESTADO DEL CM a 'Terminated' solo cambia ese campo: N CONTRATO 3PC,
+fechas, tipo y pago del CM se conservan como historial del contrato.</t>
         </is>
       </c>
       <c r="G135" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H135" s="14" t="inlineStr">
@@ -8172,37 +8170,37 @@
       </c>
       <c r="I135" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-706_CP-708 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestReglaTerminatedCm.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1427_CP-1428 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestReglaTerminatedCm.</t>
         </is>
       </c>
     </row>
     <row r="136" ht="139" customHeight="1">
-      <c r="A136" s="10" t="inlineStr">
+      <c r="A136" s="15" t="inlineStr">
         <is>
           <t>CP-709_CP-713</t>
         </is>
       </c>
-      <c r="B136" s="9" t="inlineStr">
+      <c r="B136" s="16" t="inlineStr">
         <is>
           <t>Comercial — reglas y cálculos (src/services/comercial_services.py)</t>
         </is>
       </c>
-      <c r="C136" s="9" t="inlineStr">
+      <c r="C136" s="16" t="inlineStr">
         <is>
           <t>Regla confirmada: al editar ESTADO DEL CM a 'Terminated' (en Comercial Vista Completa o en Contratos CM), se limpian a '-' N CONTRATO 3PC, FECHA INICIO CM, FECHA TERMINO CM, TIPO DE CM y PAGO CM. ESTADO DEL CM en si NO se limpia. Función pura, mismo contrato que aplica_regla_sin_contrato: no conoce pending_changes ni PyQt6.</t>
         </is>
       </c>
-      <c r="D136" s="9" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>No necesita pantallas ni archivos: son funciones de cálculo puras (pandas/Python) del módulo comercial_services. Se ejecutan junto con el resto de la batería, y también se pueden correr solas (python -m unittest src.tests.test_comercial_services).</t>
         </is>
       </c>
-      <c r="E136" s="9" t="inlineStr">
+      <c r="E136" s="16" t="inlineStr">
         <is>
           <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestAplicaReglaTerminatedCm' (archivo test_comercial_services.py). 3) Pruebas incluidas: columna distinta no hace nada; es insensible a mayusculas y espacios; running a terminated limpia cinco campos; terminated hacia otro valor no aplica regla inversa; valor nuevo no es terminated no hace nada.</t>
         </is>
       </c>
-      <c r="F136" s="9" t="inlineStr">
+      <c r="F136" s="16" t="inlineStr">
         <is>
           <t>Las 5 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada: al editar ESTADO DEL CM a 'Terminated' (en Comercial
 Vista Completa o en Contratos CM), se limpian a '-' N CONTRATO 3PC,
@@ -8211,17 +8209,17 @@
 aplica_regla_sin_contrato: no conoce pending_changes ni PyQt6.</t>
         </is>
       </c>
-      <c r="G136" s="9" t="inlineStr">
+      <c r="G136" s="16" t="inlineStr">
         <is>
           <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
-      <c r="H136" s="14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I136" s="9" t="inlineStr">
+      <c r="H136" s="17" t="inlineStr">
+        <is>
+          <t>OBSOLETA</t>
+        </is>
+      </c>
+      <c r="I136" s="16" t="inlineStr">
         <is>
           <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-709_CP-713 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial_services.py::TestAplicaReglaTerminatedCm.</t>
         </is>
@@ -8240,7 +8238,7 @@
       </c>
       <c r="C137" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: Renovaciones (y el KPI 'xvencer') se calculan en dias CALENDARIO, no habiles. Cubre los 5 casos limite explicitos: vencido, vence hoy, vence en 1 dia, vence en exactamente 30 dias (incluido) y vence en 31 dias (excluido).</t>
+          <t>Regla confirmada con Javiera: Renovaciones (y el KPI 'xvencer') se calculan en dias CALENDARIO, no habiles. Cubre los 5 casos limite explicitos: vencido, vence hoy, vence en 1 dia, vence en exactamente 30 dias (incluido) y vence en 31 dias (excluido).</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
@@ -8255,7 +8253,7 @@
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>Las 8 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con la contraparte comercial: Renovaciones (y el KPI 'xvencer') se
+          <t>Las 8 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con Javiera: Renovaciones (y el KPI 'xvencer') se
 calculan en dias CALENDARIO, no habiles. Cubre los 5 casos limite
 explicitos: vencido, vence hoy, vence en 1 dia, vence en exactamente 30
 dias (incluido) y vence en 31 dias (excluido).</t>
@@ -8263,7 +8261,7 @@
       </c>
       <c r="G137" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H137" s="14" t="inlineStr">
@@ -8315,7 +8313,7 @@
       </c>
       <c r="G138" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H138" s="14" t="inlineStr">
@@ -8342,7 +8340,7 @@
       </c>
       <c r="C139" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: ESTADO COMERCIAL == 'BAJA', igualdad exacta (nunca 'contains'), para no incluir 'BAJA SOLICITADA'.</t>
+          <t>Regla confirmada con Javiera: ESTADO COMERCIAL == 'BAJA', igualdad exacta (nunca 'contains'), para no incluir 'BAJA SOLICITADA'.</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
@@ -8364,7 +8362,7 @@
       </c>
       <c r="G139" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H139" s="14" t="inlineStr">
@@ -8391,7 +8389,7 @@
       </c>
       <c r="C140" s="9" t="inlineStr">
         <is>
-          <t>Regla confirmada con la contraparte comercial: ESTADO DE ACTIVACIÓN ACTUAL == 'NO APLICA', igualdad exacta. No debe confundirse con otros estados operacionales similares.</t>
+          <t>Regla confirmada con Javiera: ESTADO DE ACTIVACIÓN ACTUAL == 'NO APLICA', igualdad exacta. No debe confundirse con otros estados operacionales similares.</t>
         </is>
       </c>
       <c r="D140" s="9" t="inlineStr">
@@ -8406,14 +8404,14 @@
       </c>
       <c r="F140" s="9" t="inlineStr">
         <is>
-          <t>Las 2 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con la contraparte comercial: ESTADO DE ACTIVACIÓN ACTUAL == 'NO
+          <t>Las 2 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regla confirmada con Javiera: ESTADO DE ACTIVACIÓN ACTUAL == 'NO
 APLICA', igualdad exacta. No debe confundirse con otros estados
 operacionales similares.</t>
         </is>
       </c>
       <c r="G140" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H140" s="14" t="inlineStr">
@@ -8466,7 +8464,7 @@
       </c>
       <c r="G141" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 12 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H141" s="14" t="inlineStr">
@@ -8518,7 +8516,7 @@
       </c>
       <c r="G142" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H142" s="14" t="inlineStr">
@@ -8567,7 +8565,7 @@
       </c>
       <c r="G143" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H143" s="14" t="inlineStr">
@@ -8594,7 +8592,7 @@
       </c>
       <c r="C144" s="9" t="inlineStr">
         <is>
-          <t>parsear_dias_restantes() es el inverso de formatear_dias_restantes(): lo usa AppTableWidget._parse_number_like (custom_table.py) para poder ordenar 'DÍAS RESTANTES' por magnitud numérica en vez de alfabéticamente (bug reportado: ordenar esa columna no reordenaba nada).</t>
+          <t>parsear_dias_restantes() es el inverso de formatear_dias_restantes(): lo usa VolvoTableWidget._parse_number_like (custom_table.py) para poder ordenar 'DÍAS RESTANTES' por magnitud numérica en vez de alfabéticamente (bug reportado: ordenar esa columna no reordenaba nada).</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
@@ -8610,14 +8608,14 @@
       <c r="F144" s="9" t="inlineStr">
         <is>
           <t>Las 6 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: parsear_dias_restantes() es el inverso de formatear_dias_restantes():
-lo usa AppTableWidget._parse_number_like (custom_table.py) para poder
+lo usa VolvoTableWidget._parse_number_like (custom_table.py) para poder
 ordenar 'DÍAS RESTANTES' por magnitud numérica en vez de alfabéticamente
 (bug reportado: ordenar esa columna no reordenaba nada).</t>
         </is>
       </c>
       <c r="G144" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H144" s="14" t="inlineStr">
@@ -8666,7 +8664,7 @@
       </c>
       <c r="G145" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H145" s="14" t="inlineStr">
@@ -8723,7 +8721,7 @@
       </c>
       <c r="G146" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H146" s="14" t="inlineStr">
@@ -8750,7 +8748,7 @@
       </c>
       <c r="C147" s="9" t="inlineStr">
         <is>
-          <t>Ejercita el flujo real de la importación mensual 3PC (ContratosModule.importar_excel_reporte) hasta ExcelWriter.update_cells() real, contra un .xlsx y un LogApp.csv temporales -- sin mockear ExcelWriter ni la escritura real. Complementa TestContratosNoLimpiaAutomaticamenteVinAusente (que sí mockea SaveContratosThread.start y solo valida el DataFrame en memoria): aquí se comprueba que 'Contratos CM (Masivo)' realme…</t>
+          <t>Ejercita el flujo real de la importación mensual 3PC (ContratosModule.importar_excel_javiera) hasta ExcelWriter.update_cells() real, contra un .xlsx y un LogApp.csv temporales -- sin mockear ExcelWriter ni la escritura real. Complementa TestContratosNoLimpiaAutomaticamenteVinAusente (que sí mockea SaveContratosThread.start y solo valida el DataFrame en memoria): aquí se comprueba que 'Contratos CM (Masivo)' realme…</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
@@ -8766,7 +8764,7 @@
       <c r="F147" s="9" t="inlineStr">
         <is>
           <t>Las 1 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Ejercita el flujo real de la importación mensual 3PC
-(ContratosModule.importar_excel_reporte) hasta ExcelWriter.update_cells()
+(ContratosModule.importar_excel_javiera) hasta ExcelWriter.update_cells()
 real, contra un .xlsx y un LogApp.csv temporales -- sin mockear
 ExcelWriter ni la escritura real. Complementa
 TestContratosNoLimpiaAutomaticamenteVinAusente (que sí mockea
@@ -8777,7 +8775,7 @@
       </c>
       <c r="G147" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H147" s="14" t="inlineStr">
@@ -8804,7 +8802,7 @@
       </c>
       <c r="C148" s="9" t="inlineStr">
         <is>
-          <t>Regresion critica (regla confirmada con la contraparte comercial): que un VIN desaparezca del Excel mensual de CM NO debe limpiar automaticamente sus datos CM en PruebasFM. Antes de esta correccion, ContratosModule.importar_excel_reporte() ponia '-'/0.0 en los campos CM de cualquier VIN de PruebasFM que no apareciera en el archivo importado, sin ninguna revision. Este test cubre exactamente ese camino.</t>
+          <t>Regresion critica (regla confirmada con Javiera): que un VIN desaparezca del Excel mensual de CM NO debe limpiar automaticamente sus datos CM en PruebasFM. Antes de esta correccion, ContratosModule.importar_excel_javiera() ponia '-'/0.0 en los campos CM de cualquier VIN de PruebasFM que no apareciera en el archivo importado, sin ninguna revision. Este test cubre exactamente ese camino.</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
@@ -8819,17 +8817,17 @@
       </c>
       <c r="F148" s="9" t="inlineStr">
         <is>
-          <t>Las 6 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regresion critica (regla confirmada con la contraparte comercial): que un VIN
+          <t>Las 6 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Regresion critica (regla confirmada con Javiera): que un VIN
 desaparezca del Excel mensual de CM NO debe limpiar automaticamente sus
 datos CM en PruebasFM. Antes de esta correccion,
-ContratosModule.importar_excel_reporte() ponia '-'/0.0 en los campos CM
+ContratosModule.importar_excel_javiera() ponia '-'/0.0 en los campos CM
 de cualquier VIN de PruebasFM que no apareciera en el archivo importado,
 sin ninguna revision. Este test cubre exactamente ese camino.</t>
         </is>
       </c>
       <c r="G148" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H148" s="14" t="inlineStr">
@@ -8878,7 +8876,7 @@
       </c>
       <c r="G149" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H149" s="14" t="inlineStr">
@@ -8926,7 +8924,7 @@
       </c>
       <c r="G150" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H150" s="14" t="inlineStr">
@@ -8940,10 +8938,10 @@
         </is>
       </c>
     </row>
-    <row r="151" ht="179.5" customHeight="1">
+    <row r="151" ht="112" customHeight="1">
       <c r="A151" s="10" t="inlineStr">
         <is>
-          <t>CP-774_CP-776</t>
+          <t>CP-774, CP-1432</t>
         </is>
       </c>
       <c r="B151" s="9" t="inlineStr">
@@ -8963,23 +8961,20 @@
       </c>
       <c r="E151" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestContratosReglaTerminatedCm' (archivo test_contratos.py). 3) Pruebas incluidas: columna n contrato 3pc no genera columna duplicada; running a terminated limpia cinco campos; terminated a otro valor no restaura datos.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestContratosReglaTerminatedCm' (archivo test_contratos.py). 3) Pruebas incluidas: columna n contrato 3pc no genera columna duplicada; running a terminated conserva datos del cm.</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>Las 3 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Misma regla que TestReglaTerminatedCm en test_comercial.py, pero para
+          <t>Las 2 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Misma regla que TestReglaTerminatedCm en test_comercial.py, pero para
 la edición manual de ESTADO DEL CM en Contratos CM
-(ContratosModule.on_item_edited): al elegir 'Terminated' se limpian a
-'-' N CONTRATO 3PC, FECHA INICIO CM, FECHA TERMINO CM, TIPO DE CM y
-PAGO CM. No debe confundirse con la detección automática de
-cm_bajas_service.py (ausencia del VIN en el 3PC mensual): esta regla es
-manual y limpia los campos de inmediato al guardar.</t>
+(ContratosModule.on_item_edited): al elegir 'Terminated' solo cambia ese
+campo y los datos del CM se conservan como historial.</t>
         </is>
       </c>
       <c r="G151" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H151" s="14" t="inlineStr">
@@ -8989,7 +8984,7 @@
       </c>
       <c r="I151" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-774_CP-776 del Reporte de Ejecución. Test automatizado: src/tests/test_contratos.py::TestContratosReglaTerminatedCm.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-774, CP-1432 del Reporte de Ejecución. Test automatizado: src/tests/test_contratos.py::TestContratosReglaTerminatedCm.</t>
         </is>
       </c>
     </row>
@@ -9032,7 +9027,7 @@
       </c>
       <c r="G152" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H152" s="14" t="inlineStr">
@@ -9094,7 +9089,7 @@
       </c>
       <c r="G153" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H153" s="14" t="inlineStr">
@@ -9121,7 +9116,7 @@
       </c>
       <c r="C154" s="9" t="inlineStr">
         <is>
-          <t>Cambio pedido por la contraparte comercial (10-09-2026): 'Industria/s' se oculta como columna visible en Clientes (se muestra en Unidades en su lugar); 'VIN' se oculta como columna visible en Unidades (sigue en el DataFrame base y sigue siendo buscable vía el buscador global de MainWindow); 'ETAPA GESTIÓN' se agrega como columna visible en Unidades, coloreada reutilizando exactamente los colores que MODULE_COLORS (colors.py) ya as…</t>
+          <t>Cambio pedido por Javiera (10-09-2026): 'Industria/s' se oculta como columna visible en Clientes (se muestra en Unidades en su lugar); 'VIN' se oculta como columna visible en Unidades (sigue en el DataFrame base y sigue siendo buscable vía el buscador global de MainWindow); 'ETAPA GESTIÓN' se agrega como columna visible en Unidades, coloreada reutilizando exactamente los colores que MODULE_COLORS (colors.py) ya as…</t>
         </is>
       </c>
       <c r="D154" s="9" t="inlineStr">
@@ -9151,7 +9146,7 @@
       </c>
       <c r="G154" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H154" s="14" t="inlineStr">
@@ -9201,7 +9196,7 @@
       </c>
       <c r="G155" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H155" s="14" t="inlineStr">
@@ -9251,7 +9246,7 @@
       </c>
       <c r="G156" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H156" s="14" t="inlineStr">
@@ -9307,7 +9302,7 @@
       </c>
       <c r="G157" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H157" s="14" t="inlineStr">
@@ -9358,7 +9353,7 @@
       </c>
       <c r="G158" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H158" s="14" t="inlineStr">
@@ -9409,7 +9404,7 @@
       </c>
       <c r="G159" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H159" s="14" t="inlineStr">
@@ -9457,7 +9452,7 @@
       </c>
       <c r="G160" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H160" s="14" t="inlineStr">
@@ -9506,7 +9501,7 @@
       </c>
       <c r="G161" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H161" s="14" t="inlineStr">
@@ -9554,7 +9549,7 @@
       </c>
       <c r="G162" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H162" s="14" t="inlineStr">
@@ -9601,7 +9596,7 @@
       </c>
       <c r="G163" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H163" s="14" t="inlineStr">
@@ -9649,7 +9644,7 @@
       </c>
       <c r="G164" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H164" s="14" t="inlineStr">
@@ -9696,7 +9691,7 @@
       </c>
       <c r="G165" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H165" s="14" t="inlineStr">
@@ -9743,7 +9738,7 @@
       </c>
       <c r="G166" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H166" s="14" t="inlineStr">
@@ -9760,7 +9755,7 @@
     <row r="167" ht="300" customHeight="1">
       <c r="A167" s="10" t="inlineStr">
         <is>
-          <t>CP-838_CP-844</t>
+          <t>CP-838_CP-839, CP-842_CP-844, CP-1422_CP-1423</t>
         </is>
       </c>
       <c r="B167" s="9" t="inlineStr">
@@ -9780,7 +9775,7 @@
       </c>
       <c r="E167" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestAgregarContactoComercial' (archivo test_comercial.py). 3) Pruebas incluidas: 01 sin seleccion boton deshabilitado; 02 multiples vin boton deshabilitado; 03 un vin con cdb con contacto boton azul; 04 un vin con cdb sin contacto boton rojo; 05 clic abre contactosadddialog con cdb y razon social correctos; 06 guardar usa addcontactothread con el writer y el id generado; … (y 1 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestAgregarContactoComercial' (archivo test_comercial.py). 3) Pruebas incluidas: 01 sin seleccion boton deshabilitado; 02 multiples vin boton deshabilitado; 03 un vin con cdb con contacto icono verde; 04 un vin con cdb sin contacto icono rojo; 05 clic abre contactosadddialog con cdb y razon social correctos; 06 guardar usa addcontactothread con el writer y el id generado; … (y 1 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F167" s="9" t="inlineStr">
@@ -9803,7 +9798,7 @@
       </c>
       <c r="G167" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H167" s="14" t="inlineStr">
@@ -9813,7 +9808,7 @@
       </c>
       <c r="I167" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-838_CP-844 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestAgregarContactoComercial.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-838_CP-839, CP-842_CP-844, CP-1422_CP-1423 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestAgregarContactoComercial.</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9855,7 @@
       </c>
       <c r="G168" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H168" s="14" t="inlineStr">
@@ -9874,10 +9869,10 @@
         </is>
       </c>
     </row>
-    <row r="169" ht="193" customHeight="1">
+    <row r="169" ht="220" customHeight="1">
       <c r="A169" s="10" t="inlineStr">
         <is>
-          <t>CP-850_CP-852</t>
+          <t>CP-852, CP-1424_CP-1425</t>
         </is>
       </c>
       <c r="B169" s="9" t="inlineStr">
@@ -9897,7 +9892,7 @@
       </c>
       <c r="E169" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestEnviarCorreoOtrasSubpestanas' (archivo test_comercial.py). 3) Pruebas incluidas: 01 un vin abre mail dialog sin plantilla preseleccionada; 02 multiples vin se entregan todos sin plantilla; 03 gestionar cm conserva su plantilla preseleccionada.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestEnviarCorreoOtrasSubpestanas' (archivo test_comercial.py). 3) Pruebas incluidas: 01 un vin abre mail dialog con conoce volvo connect preseleccionada; 02 multiples vin se entregan todos con su plantilla; 03 gestionar cm conserva su plantilla preseleccionada.</t>
         </is>
       </c>
       <c r="F169" s="9" t="inlineStr">
@@ -9907,13 +9902,14 @@
 _on_accion_cm_enviar_correo_clicked y _obtener_vins_seleccionados):
 mismo flujo que en "Gestionar CM" (TestEnviarCorreoCM), pero resolviendo
 la selección contra _new_ui_bandeja_actual_df (subset de df_base) en vez
-de _new_ui_revision_cm_df, y SIN plantilla preseleccionada. No abre un
+de _new_ui_revision_cm_df, con "Conoce Volvo Connect" preseleccionada
+(Nuevas oportunidades, 21-10-2026; antes sin plantilla). No abre un
 MailDialog real: parchea MailDialog y el chequeo de VIN faltantes.</t>
         </is>
       </c>
       <c r="G169" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H169" s="14" t="inlineStr">
@@ -9923,7 +9919,7 @@
       </c>
       <c r="I169" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-850_CP-852 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestEnviarCorreoOtrasSubpestanas.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-852, CP-1424_CP-1425 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestEnviarCorreoOtrasSubpestanas.</t>
         </is>
       </c>
     </row>
@@ -9969,7 +9965,7 @@
       </c>
       <c r="G170" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H170" s="14" t="inlineStr">
@@ -10021,7 +10017,7 @@
       </c>
       <c r="G171" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H171" s="14" t="inlineStr">
@@ -10080,7 +10076,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H172" s="14" t="inlineStr">
@@ -10131,7 +10127,7 @@
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H173" s="14" t="inlineStr">
@@ -10182,7 +10178,7 @@
       </c>
       <c r="G174" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H174" s="14" t="inlineStr">
@@ -10234,7 +10230,7 @@
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H175" s="14" t="inlineStr">
@@ -10284,7 +10280,7 @@
       </c>
       <c r="G176" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 16 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 16 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H176" s="14" t="inlineStr">
@@ -10337,7 +10333,7 @@
       </c>
       <c r="G177" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H177" s="14" t="inlineStr">
@@ -10392,12 +10388,12 @@
       </c>
       <c r="G178" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 33 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
-        </is>
-      </c>
-      <c r="H178" s="14" t="inlineStr">
-        <is>
-          <t>PASS</t>
+          <t>31 de 33 aprobadas, 2 falladas (FAIL), 0 con error (ERROR) en la ejecución del 22-10-2026 12:36:02. Revisar el Reporte de Defectos.</t>
+        </is>
+      </c>
+      <c r="H178" s="19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I178" s="9" t="inlineStr">
@@ -10449,7 +10445,7 @@
       </c>
       <c r="G179" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H179" s="14" t="inlineStr">
@@ -10500,7 +10496,7 @@
       </c>
       <c r="G180" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H180" s="14" t="inlineStr">
@@ -10556,7 +10552,7 @@
       </c>
       <c r="G181" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H181" s="14" t="inlineStr">
@@ -10612,7 +10608,7 @@
       </c>
       <c r="G182" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H182" s="14" t="inlineStr">
@@ -10669,7 +10665,7 @@
       </c>
       <c r="G183" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 21 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 21 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H183" s="14" t="inlineStr">
@@ -10720,7 +10716,7 @@
       </c>
       <c r="G184" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H184" s="14" t="inlineStr">
@@ -10771,7 +10767,7 @@
       </c>
       <c r="G185" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H185" s="14" t="inlineStr">
@@ -10821,7 +10817,7 @@
       </c>
       <c r="G186" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H186" s="14" t="inlineStr">
@@ -10870,7 +10866,7 @@
       </c>
       <c r="G187" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H187" s="14" t="inlineStr">
@@ -10917,7 +10913,7 @@
       </c>
       <c r="G188" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H188" s="14" t="inlineStr">
@@ -10964,7 +10960,7 @@
       </c>
       <c r="G189" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H189" s="14" t="inlineStr">
@@ -11011,7 +11007,7 @@
       </c>
       <c r="G190" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H190" s="14" t="inlineStr">
@@ -11038,7 +11034,7 @@
       </c>
       <c r="C191" s="9" t="inlineStr">
         <is>
-          <t>Plantilla base de Facturación Manual (fase 'Crear plantilla base', ver facturacionManual.txt): solo estructura visual, sin cálculos ni conexión a 'Facturación Manual - BBDD.xlsx'. Todo campo financiero debe quedar literalmente marcado como PENDIENTE CONTRAPARTE COMERCIAL.</t>
+          <t>Plantilla base de Facturación Manual (fase 'Crear plantilla base', ver facturacionManual.txt): solo estructura visual, sin cálculos ni conexión a 'Facturación Manual - BBDD.xlsx'. Todo campo financiero debe quedar literalmente marcado como PENDIENTE JAVIERA.</t>
         </is>
       </c>
       <c r="D191" s="9" t="inlineStr">
@@ -11054,14 +11050,14 @@
       <c r="F191" s="9" t="inlineStr">
         <is>
           <t>Las 5 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Plantilla base de Facturación Manual (fase 'Crear plantilla base', ver
-facturacionManual.txt): solo estructura visual, sin cálculos ni conexión
+Notas del proyecto.txt, sección 7): solo estructura visual, sin cálculos ni conexión
 a 'Facturación Manual - BBDD.xlsx'. Todo campo financiero debe quedar
-literalmente marcado como PENDIENTE CONTRAPARTE COMERCIAL.</t>
+literalmente marcado como PENDIENTE JAVIERA.</t>
         </is>
       </c>
       <c r="G191" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H191" s="14" t="inlineStr">
@@ -11108,7 +11104,7 @@
       </c>
       <c r="G192" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H192" s="14" t="inlineStr">
@@ -11156,7 +11152,7 @@
       </c>
       <c r="G193" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H193" s="14" t="inlineStr">
@@ -11205,7 +11201,7 @@
       </c>
       <c r="G194" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H194" s="14" t="inlineStr">
@@ -11253,7 +11249,7 @@
       </c>
       <c r="G195" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H195" s="14" t="inlineStr">
@@ -11302,7 +11298,7 @@
       </c>
       <c r="G196" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H196" s="14" t="inlineStr">
@@ -11362,7 +11358,7 @@
       </c>
       <c r="G197" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H197" s="14" t="inlineStr">
@@ -11475,7 +11471,7 @@
       </c>
       <c r="G199" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H199" s="14" t="inlineStr">
@@ -11526,7 +11522,7 @@
       </c>
       <c r="G200" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H200" s="14" t="inlineStr">
@@ -11647,7 +11643,7 @@
       </c>
       <c r="G202" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 10 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H202" s="14" t="inlineStr">
@@ -11702,7 +11698,7 @@
       </c>
       <c r="G203" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H203" s="14" t="inlineStr">
@@ -11754,7 +11750,7 @@
       </c>
       <c r="G204" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H204" s="14" t="inlineStr">
@@ -11808,7 +11804,7 @@
       </c>
       <c r="G205" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H205" s="14" t="inlineStr">
@@ -11865,7 +11861,7 @@
       </c>
       <c r="G206" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H206" s="14" t="inlineStr">
@@ -11916,7 +11912,7 @@
       </c>
       <c r="G207" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H207" s="14" t="inlineStr">
@@ -11965,7 +11961,7 @@
       </c>
       <c r="G208" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H208" s="14" t="inlineStr">
@@ -12020,7 +12016,7 @@
       </c>
       <c r="G209" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H209" s="14" t="inlineStr">
@@ -12069,7 +12065,7 @@
       </c>
       <c r="G210" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H210" s="14" t="inlineStr">
@@ -12116,7 +12112,7 @@
       </c>
       <c r="G211" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H211" s="14" t="inlineStr">
@@ -12174,7 +12170,7 @@
       </c>
       <c r="G212" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 9 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H212" s="14" t="inlineStr">
@@ -12227,7 +12223,7 @@
       </c>
       <c r="G213" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H213" s="14" t="inlineStr">
@@ -12338,7 +12334,7 @@
       </c>
       <c r="G215" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H215" s="14" t="inlineStr">
@@ -12392,7 +12388,7 @@
       </c>
       <c r="G216" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 8 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H216" s="14" t="inlineStr">
@@ -12442,7 +12438,7 @@
       </c>
       <c r="G217" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H217" s="14" t="inlineStr">
@@ -12494,7 +12490,7 @@
       </c>
       <c r="G218" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H218" s="14" t="inlineStr">
@@ -12545,7 +12541,7 @@
       </c>
       <c r="G219" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H219" s="14" t="inlineStr">
@@ -12572,7 +12568,7 @@
       </c>
       <c r="C220" s="9" t="inlineStr">
         <is>
-          <t>24-09-2026, a pedido explícito: tras sincronizar, RMReporteSyncWorker debe: (1) normalizar automáticamente TIPO DE FACTURACION cuando está sin asignar y la matriz tiene una única opción válida (escribe a PruebasFM.csv); (2) avisar -- solo informativo, nunca corregir -- cuántas combinaciones reales quedan incompatibles con la matriz; (3) avisar cuántas unidades siguen sin asignar porque la matriz permite más de una op…</t>
+          <t>24-09-2026, a pedido explícito: tras sincronizar, RMJaviSyncWorker debe: (1) normalizar automáticamente TIPO DE FACTURACION cuando está sin asignar y la matriz tiene una única opción válida (escribe a PruebasFM.csv); (2) avisar -- solo informativo, nunca corregir -- cuántas combinaciones reales quedan incompatibles con la matriz; (3) avisar cuántas unidades siguen sin asignar porque la matriz permite más de una op…</t>
         </is>
       </c>
       <c r="D220" s="9" t="inlineStr">
@@ -12582,15 +12578,15 @@
       </c>
       <c r="E220" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMReporteSyncValidacionFormaContratoTipoFacturacion' (archivo test_comercial.py). 3) Pruebas incluidas: forma de contrato con multiples opciones no se toca; forma de contrato con una sola opcion se normaliza en el csv final; log en vivo incluye avisos; mensaje final incluye conteo de inconsistencias reales; mensaje final incluye conteo de normalizados; mensaje final incluye conteo de sin asignar; … (y 1 más, ver el Reporte de Ejecución).</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMJaviSyncValidacionFormaContratoTipoFacturacion' (archivo test_comercial.py). 3) Pruebas incluidas: forma de contrato con multiples opciones no se toca; forma de contrato con una sola opcion se normaliza en el csv final; log en vivo incluye avisos; mensaje final incluye conteo de inconsistencias reales; mensaje final incluye conteo de normalizados; mensaje final incluye conteo de sin asignar; … (y 1 más, ver el Reporte de Ejecución).</t>
         </is>
       </c>
       <c r="F220" s="9" t="inlineStr">
         <is>
-          <t>Las 7 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: 24-09-2026, a pedido explícito: tras sincronizar, RMReporteSyncWorker debe:
+          <t>Las 7 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: 24-09-2026, a pedido explícito: tras sincronizar, RMJaviSyncWorker debe:
 (1) normalizar automáticamente TIPO DE FACTURACION cuando está sin
 asignar y la matriz tiene una única opción válida (escribe a
-RM_CONTRATOS.csv); (2) avisar -- solo informativo, nunca corregir -- cuántas
+RM_JAVI.csv); (2) avisar -- solo informativo, nunca corregir -- cuántas
 combinaciones reales quedan incompatibles con la matriz; (3) avisar
 cuántas unidades siguen sin asignar porque la matriz permite más de una
 opción. Reutiliza tal cual comercial_services.detectar_inconsistencias_
@@ -12601,7 +12597,7 @@
       </c>
       <c r="G220" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H220" s="14" t="inlineStr">
@@ -12611,7 +12607,7 @@
       </c>
       <c r="I220" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1223_CP-1229 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMReporteSyncValidacionFormaContratoTipoFacturacion.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1223_CP-1229 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial.py::TestRMJaviSyncValidacionFormaContratoTipoFacturacion.</t>
         </is>
       </c>
     </row>
@@ -12650,7 +12646,7 @@
       </c>
       <c r="G221" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H221" s="14" t="inlineStr">
@@ -12701,7 +12697,7 @@
       </c>
       <c r="G222" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H222" s="14" t="inlineStr">
@@ -12750,7 +12746,7 @@
       </c>
       <c r="G223" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 15 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H223" s="14" t="inlineStr">
@@ -12777,7 +12773,7 @@
       </c>
       <c r="C224" s="9" t="inlineStr">
         <is>
-          <t>detectar_inconsistencias_forma_contrato_tipo_facturacion() reutiliza FORMA_CONTRATO_TIPO_FACTURACION_MATRIZ (constants.py, matriz de la contraparte comercial, 24-09-2026) como única fuente de verdad -- misma matriz que ya aplica en vivo ComercialAgregarDialog. Es una herramienta de solo DETECCIÓN para datos históricos: nunca modifica ninguna fila.</t>
+          <t>detectar_inconsistencias_forma_contrato_tipo_facturacion() reutiliza FORMA_CONTRATO_TIPO_FACTURACION_MATRIZ (constants.py, matriz de Javiera, 24-09-2026) como única fuente de verdad -- misma matriz que ya aplica en vivo ComercialAgregarDialog. Es una herramienta de solo DETECCIÓN para datos históricos: nunca modifica ninguna fila.</t>
         </is>
       </c>
       <c r="D224" s="9" t="inlineStr">
@@ -12793,7 +12789,7 @@
       <c r="F224" s="9" t="inlineStr">
         <is>
           <t>Las 13 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: detectar_inconsistencias_forma_contrato_tipo_facturacion() reutiliza
-FORMA_CONTRATO_TIPO_FACTURACION_MATRIZ (constants.py, matriz de la contraparte comercial,
+FORMA_CONTRATO_TIPO_FACTURACION_MATRIZ (constants.py, matriz de Javiera,
 24-09-2026) como única fuente de verdad -- misma matriz que ya aplica en
 vivo ComercialAgregarDialog. Es una herramienta de solo DETECCIÓN para
 datos históricos: nunca modifica ninguna fila.</t>
@@ -12801,7 +12797,7 @@
       </c>
       <c r="G224" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 13 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H224" s="14" t="inlineStr">
@@ -12852,7 +12848,7 @@
       </c>
       <c r="G225" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 18 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 18 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H225" s="14" t="inlineStr">
@@ -12879,7 +12875,7 @@
       </c>
       <c r="C226" s="9" t="inlineStr">
         <is>
-          <t>Actualizado (30-09-2026, a pedido explícito): la regla que forzaba 'PROVISION +' a DURACIÓN (MESES)='-' / TÉRMINO CONTRATO='MENSUAL' sin excepción se desactivó (ver dataframe_formatter.py). RM_CONTRATOS siempre trae una fecha real de término para estas filas; la regla la sobrescribía y ocultaba contratos ya caducados (391 de 561 filas reales al momento de desactivarla). 'PROVISION +' ahora sigue exactamente la misma re…</t>
+          <t>Actualizado (30-09-2026, a pedido explícito): la regla que forzaba 'PROVISION +' a DURACIÓN (MESES)='-' / TÉRMINO CONTRATO='MENSUAL' sin excepción se desactivó (ver dataframe_formatter.py). RM_JAVI siempre trae una fecha real de término para estas filas; la regla la sobrescribía y ocultaba contratos ya caducados (391 de 561 filas reales al momento de desactivarla). 'PROVISION +' ahora sigue exactamente la misma re…</t>
         </is>
       </c>
       <c r="D226" s="9" t="inlineStr">
@@ -12896,7 +12892,7 @@
         <is>
           <t>Las 7 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Actualizado (30-09-2026, a pedido explícito): la regla que forzaba
 'PROVISION +' a DURACIÓN (MESES)='-' / TÉRMINO CONTRATO='MENSUAL' sin
-excepción se desactivó (ver dataframe_formatter.py). RM_CONTRATOS siempre trae
+excepción se desactivó (ver dataframe_formatter.py). RM_JAVI siempre trae
 una fecha real de término para estas filas; la regla la sobrescribía y
 ocultaba contratos ya caducados (391 de 561 filas reales al momento de
 desactivarla). 'PROVISION +' ahora sigue exactamente la misma regla
@@ -12907,7 +12903,7 @@
       </c>
       <c r="G226" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H226" s="14" t="inlineStr">
@@ -12954,7 +12950,7 @@
       </c>
       <c r="G227" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H227" s="14" t="inlineStr">
@@ -13001,7 +12997,7 @@
       </c>
       <c r="G228" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H228" s="14" t="inlineStr">
@@ -13052,7 +13048,7 @@
       </c>
       <c r="G229" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H229" s="14" t="inlineStr">
@@ -13099,7 +13095,7 @@
       </c>
       <c r="G230" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H230" s="14" t="inlineStr">
@@ -13146,7 +13142,7 @@
       </c>
       <c r="G231" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H231" s="14" t="inlineStr">
@@ -13193,7 +13189,7 @@
       </c>
       <c r="G232" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H232" s="14" t="inlineStr">
@@ -13240,7 +13236,7 @@
       </c>
       <c r="G233" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 1 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H233" s="14" t="inlineStr">
@@ -13288,7 +13284,7 @@
       </c>
       <c r="G234" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H234" s="14" t="inlineStr">
@@ -13315,7 +13311,7 @@
       </c>
       <c r="C235" s="9" t="inlineStr">
         <is>
-          <t>Misma secuencia (merge/limpieza/logging real, sin mocks de negocio) que TestRMReporteSyncActualizaHistorial (test_comercial.py), pero comparando el resultado contra un PruebasFM destino .xlsx y uno .csv.</t>
+          <t>Misma secuencia (merge/limpieza/logging real, sin mocks de negocio) que TestRMJaviSyncActualizaHistorial (test_comercial.py), pero comparando el resultado contra un PruebasFM destino .xlsx y uno .csv.</t>
         </is>
       </c>
       <c r="D235" s="9" t="inlineStr">
@@ -13325,19 +13321,19 @@
       </c>
       <c r="E235" s="9" t="inlineStr">
         <is>
-          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMReporteSyncCsvVsXlsx' (archivo test_fase2_csv_integration.py). 3) Pruebas incluidas: equivalencia df final xlsx vs csv; sync contra csv escribe dataset completo; sync contra xlsx escribe y conserva estructura.</t>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestRMJaviSyncCsvVsXlsx' (archivo test_fase2_csv_integration.py). 3) Pruebas incluidas: equivalencia df final xlsx vs csv; sync contra csv escribe dataset completo; sync contra xlsx escribe y conserva estructura.</t>
         </is>
       </c>
       <c r="F235" s="9" t="inlineStr">
         <is>
           <t>Las 3 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Misma secuencia (merge/limpieza/logging real, sin mocks de negocio)
-que TestRMReporteSyncActualizaHistorial (test_comercial.py), pero comparando
+que TestRMJaviSyncActualizaHistorial (test_comercial.py), pero comparando
 el resultado contra un PruebasFM destino .xlsx y uno .csv.</t>
         </is>
       </c>
       <c r="G235" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H235" s="14" t="inlineStr">
@@ -13347,7 +13343,7 @@
       </c>
       <c r="I235" s="9" t="inlineStr">
         <is>
-          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1350_CP-1352 del Reporte de Ejecución. Test automatizado: src/tests/test_fase2_csv_integration.py::TestRMReporteSyncCsvVsXlsx.</t>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1350_CP-1352 del Reporte de Ejecución. Test automatizado: src/tests/test_fase2_csv_integration.py::TestRMJaviSyncCsvVsXlsx.</t>
         </is>
       </c>
     </row>
@@ -13388,7 +13384,7 @@
       </c>
       <c r="G236" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H236" s="14" t="inlineStr">
@@ -13435,7 +13431,7 @@
       </c>
       <c r="G237" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H237" s="14" t="inlineStr">
@@ -13482,7 +13478,7 @@
       </c>
       <c r="G238" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H238" s="14" t="inlineStr">
@@ -13529,7 +13525,7 @@
       </c>
       <c r="G239" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H239" s="14" t="inlineStr">
@@ -13577,7 +13573,7 @@
       </c>
       <c r="G240" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 3 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H240" s="14" t="inlineStr">
@@ -13627,7 +13623,7 @@
       </c>
       <c r="G241" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 5 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H241" s="14" t="inlineStr">
@@ -13675,7 +13671,7 @@
       </c>
       <c r="G242" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H242" s="14" t="inlineStr">
@@ -13725,7 +13721,7 @@
       </c>
       <c r="G243" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 7 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H243" s="14" t="inlineStr">
@@ -13773,7 +13769,7 @@
       </c>
       <c r="G244" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 6 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H244" s="14" t="inlineStr">
@@ -13821,7 +13817,7 @@
       </c>
       <c r="G245" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H245" s="14" t="inlineStr">
@@ -13870,7 +13866,7 @@
       </c>
       <c r="G246" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 4 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H246" s="14" t="inlineStr">
@@ -13918,7 +13914,7 @@
       </c>
       <c r="G247" s="9" t="inlineStr">
         <is>
-          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 13-10-2026 13:01:16. Detalle en el Reporte de Ejecución de Pruebas.</t>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
         </is>
       </c>
       <c r="H247" s="14" t="inlineStr">
@@ -13932,8 +13928,56 @@
         </is>
       </c>
     </row>
+    <row r="248" ht="85" customHeight="1">
+      <c r="A248" s="10" t="inlineStr">
+        <is>
+          <t>CP-1429_CP-1430</t>
+        </is>
+      </c>
+      <c r="B248" s="9" t="inlineStr">
+        <is>
+          <t>Dataframe Formatter — núcleo (src/core/dataframe_formatter.py)</t>
+        </is>
+      </c>
+      <c r="C248" s="9" t="inlineStr">
+        <is>
+          <t>Contratos (CM) no muestra ningún contrato en Baja o Baja solicitada, aunque la unidad siga conectada.</t>
+        </is>
+      </c>
+      <c r="D248" s="9" t="inlineStr">
+        <is>
+          <t>No necesita pantallas ni archivos: son funciones de cálculo puras (pandas/Python) del módulo comercial_services. Se ejecutan junto con el resto de la batería, y también se pueden correr solas (python -m unittest src.tests.test_comercial_services).</t>
+        </is>
+      </c>
+      <c r="E248" s="9" t="inlineStr">
+        <is>
+          <t>1) Ejecutar la batería completa (python src/tests/auditor/run_auditor.py). 2) El sistema corre el grupo de pruebas 'TestExcluirContratosCerrados' (archivo test_comercial_services.py). 3) Pruebas incluidas: quita baja y baja solicitada aunque sigan conectados; sin columna o vacio devuelve igual.</t>
+        </is>
+      </c>
+      <c r="F248" s="9" t="inlineStr">
+        <is>
+          <t>Las 2 prueba(s) del grupo terminan en PASS (aprobadas). Qué se verifica: Contratos (CM) no muestra ningún contrato en Baja o Baja solicitada,
+aunque la unidad siga conectada.</t>
+        </is>
+      </c>
+      <c r="G248" s="9" t="inlineStr">
+        <is>
+          <t>PASS: las 2 prueba(s) se aprobaron en la ejecución del 22-10-2026 12:36:02. Detalle en el Reporte de Ejecución de Pruebas.</t>
+        </is>
+      </c>
+      <c r="H248" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I248" s="9" t="inlineStr">
+        <is>
+          <t>Generado por el auditor automático (src/tests/auditor/run_auditor.py). Casos CP-1429_CP-1430 del Reporte de Ejecución. Test automatizado: src/tests/test_comercial_services.py::TestExcluirContratosCerrados.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I247"/>
+  <autoFilter ref="A1:I248"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>